<commit_message>
Robustify matrix_to_table; add outputs and logs
Update R/01_utils.R: make matrix_to_table resilient to NULLs, atomic vectors, data.frames and zero-dimension objects; convert inputs safely to matrices, preserve row names, and return an empty tibble for invalid input. Add many generated output artifacts from a pipeline run: new correlation figures, updated figure/table binaries, outputs/logs/transformation_audit_log.csv, outputs/models/cfa_competence_second_order_summary.txt, and new data-quality/sample-audit spreadsheets. .Rhistory also reflects the pipeline run.
</commit_message>
<xml_diff>
--- a/outputs/tables/cfa_results.xlsx
+++ b/outputs/tables/cfa_results.xlsx
@@ -17,17 +17,29 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="98">
   <si>
     <t xml:space="preserve">model</t>
   </si>
   <si>
+    <t xml:space="preserve">sample</t>
+  </si>
+  <si>
     <t xml:space="preserve">converged</t>
   </si>
   <si>
+    <t xml:space="preserve">post_estimation_check</t>
+  </si>
+  <si>
     <t xml:space="preserve">admissible_solution</t>
   </si>
   <si>
+    <t xml:space="preserve">n_used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">free_parameters</t>
+  </si>
+  <si>
     <t xml:space="preserve">min_eigenvalue_latent_covariance</t>
   </si>
   <si>
@@ -38,6 +50,9 @@
   </si>
   <si>
     <t xml:space="preserve">GAAIS: correlated Positive and NegativeFavorable factors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full sample</t>
   </si>
   <si>
     <t xml:space="preserve">AI Literacy: four correlated factors</t>
@@ -97,13 +112,13 @@
     <t xml:space="preserve">standardized_loading</t>
   </si>
   <si>
-    <t xml:space="preserve">se</t>
-  </si>
-  <si>
-    <t xml:space="preserve">z</t>
-  </si>
-  <si>
-    <t xml:space="preserve">p</t>
+    <t xml:space="preserve">standard_error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">z_value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p_value</t>
   </si>
   <si>
     <t xml:space="preserve">Positive</t>
@@ -244,6 +259,12 @@
     <t xml:space="preserve">items</t>
   </si>
   <si>
+    <t xml:space="preserve">usable_items</t>
+  </si>
+  <si>
+    <t xml:space="preserve">removed_zero_variance_items</t>
+  </si>
+  <si>
     <t xml:space="preserve">kmo_overall</t>
   </si>
   <si>
@@ -286,7 +307,10 @@
     <t xml:space="preserve">GAAIS two-factor item set</t>
   </si>
   <si>
-    <t xml:space="preserve">CFA is applicable; model adequacy still depends on convergence, admissibility, fit, and theoretically coherent loadings.</t>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
+    <t xml:space="preserve">CFA is applicable. Interpret fit, loadings, residuals, factor correlations, and theory jointly.</t>
   </si>
   <si>
     <t xml:space="preserve">AI Literacy four-factor item set</t>
@@ -337,64 +361,71 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:F4" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:F4"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:J4" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:J4"/>
+  <tableColumns count="10">
     <tableColumn id="1" name="model"/>
-    <tableColumn id="2" name="converged"/>
-    <tableColumn id="3" name="admissible_solution"/>
-    <tableColumn id="4" name="min_eigenvalue_latent_covariance"/>
-    <tableColumn id="5" name="error"/>
-    <tableColumn id="6" name="warnings"/>
+    <tableColumn id="2" name="sample"/>
+    <tableColumn id="3" name="converged"/>
+    <tableColumn id="4" name="post_estimation_check"/>
+    <tableColumn id="5" name="admissible_solution"/>
+    <tableColumn id="6" name="n_used"/>
+    <tableColumn id="7" name="free_parameters"/>
+    <tableColumn id="8" name="min_eigenvalue_latent_covariance"/>
+    <tableColumn id="9" name="error"/>
+    <tableColumn id="10" name="warnings"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Table4" displayName="Table4" ref="A1:C28" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:C28"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Table4" displayName="Table4" ref="A1:D28" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:D28"/>
+  <tableColumns count="4">
     <tableColumn id="1" name="model"/>
-    <tableColumn id="2" name="measure"/>
-    <tableColumn id="3" name="value"/>
+    <tableColumn id="2" name="sample"/>
+    <tableColumn id="3" name="measure"/>
+    <tableColumn id="4" name="value"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Table5" displayName="Table5" ref="A1:G33" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:G33"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Table5" displayName="Table5" ref="A1:H33" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:H33"/>
+  <tableColumns count="8">
     <tableColumn id="1" name="model"/>
-    <tableColumn id="2" name="factor"/>
-    <tableColumn id="3" name="item"/>
-    <tableColumn id="4" name="standardized_loading"/>
-    <tableColumn id="5" name="se"/>
-    <tableColumn id="6" name="z"/>
-    <tableColumn id="7" name="p"/>
+    <tableColumn id="2" name="sample"/>
+    <tableColumn id="3" name="factor"/>
+    <tableColumn id="4" name="item"/>
+    <tableColumn id="5" name="standardized_loading"/>
+    <tableColumn id="6" name="standard_error"/>
+    <tableColumn id="7" name="z_value"/>
+    <tableColumn id="8" name="p_value"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Table6" displayName="Table6" ref="A1:D8" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:D8"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Table6" displayName="Table6" ref="A1:E21" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E21"/>
+  <tableColumns count="5">
     <tableColumn id="1" name="model"/>
-    <tableColumn id="2" name="factor_1"/>
-    <tableColumn id="3" name="factor_2"/>
-    <tableColumn id="4" name="correlation"/>
+    <tableColumn id="2" name="sample"/>
+    <tableColumn id="3" name="factor_1"/>
+    <tableColumn id="4" name="factor_2"/>
+    <tableColumn id="5" name="correlation"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Table7" displayName="Table7" ref="A1:D3" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:D3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Table7" displayName="Table7" ref="A1:D5" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:D5"/>
   <tableColumns count="4">
     <tableColumn id="1" name="model"/>
     <tableColumn id="2" name="factor"/>
@@ -406,25 +437,27 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Table8" displayName="Table8" ref="A1:P3" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:P3"/>
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Table8" displayName="Table8" ref="A1:R3" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:R3"/>
+  <tableColumns count="18">
     <tableColumn id="1" name="scale"/>
     <tableColumn id="2" name="n_complete"/>
     <tableColumn id="3" name="items"/>
-    <tableColumn id="4" name="kmo_overall"/>
-    <tableColumn id="5" name="bartlett_chisq"/>
-    <tableColumn id="6" name="bartlett_df"/>
-    <tableColumn id="7" name="bartlett_p"/>
-    <tableColumn id="8" name="min_item_variance"/>
-    <tableColumn id="9" name="max_absolute_item_correlation"/>
-    <tableColumn id="10" name="sample_to_item_ratio"/>
-    <tableColumn id="11" name="kmo_adequate"/>
-    <tableColumn id="12" name="bartlett_significant"/>
-    <tableColumn id="13" name="item_variance_adequate"/>
-    <tableColumn id="14" name="sample_size_adequate"/>
-    <tableColumn id="15" name="cfa_applicable"/>
-    <tableColumn id="16" name="interpretation"/>
+    <tableColumn id="4" name="usable_items"/>
+    <tableColumn id="5" name="removed_zero_variance_items"/>
+    <tableColumn id="6" name="kmo_overall"/>
+    <tableColumn id="7" name="bartlett_chisq"/>
+    <tableColumn id="8" name="bartlett_df"/>
+    <tableColumn id="9" name="bartlett_p"/>
+    <tableColumn id="10" name="min_item_variance"/>
+    <tableColumn id="11" name="max_absolute_item_correlation"/>
+    <tableColumn id="12" name="sample_to_item_ratio"/>
+    <tableColumn id="13" name="kmo_adequate"/>
+    <tableColumn id="14" name="bartlett_significant"/>
+    <tableColumn id="15" name="item_variance_adequate"/>
+    <tableColumn id="16" name="sample_size_adequate"/>
+    <tableColumn id="17" name="cfa_applicable"/>
+    <tableColumn id="18" name="interpretation"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -713,11 +746,15 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="56.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="9.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="19.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="32.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="5.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="245.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="11.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="9.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="21.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="19.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="6.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="15.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="32.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="5.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="245.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -739,57 +776,105 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="b">
-        <v>1</v>
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1211</v>
+      </c>
+      <c r="G2" t="n">
+        <v>101</v>
+      </c>
+      <c r="H2" t="n">
         <v>0.941848216725088</v>
       </c>
-      <c r="E2"/>
-      <c r="F2"/>
+      <c r="I2"/>
+      <c r="J2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="b">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="b">
         <v>1</v>
       </c>
-      <c r="C3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
+      <c r="D3" t="b">
+        <v>0</v>
+      </c>
+      <c r="E3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1211</v>
+      </c>
+      <c r="G3" t="n">
+        <v>66</v>
+      </c>
+      <c r="H3" t="n">
         <v>-0.0462482493018743</v>
       </c>
-      <c r="E3"/>
-      <c r="F3" t="s">
-        <v>8</v>
+      <c r="I3"/>
+      <c r="J3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="b">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
       </c>
       <c r="C4" t="b">
         <v>0</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1211</v>
+      </c>
+      <c r="G4" t="n">
+        <v>64</v>
+      </c>
+      <c r="H4" t="n">
         <v>0.000000481633461668629</v>
       </c>
-      <c r="E4"/>
-      <c r="F4" t="s">
-        <v>10</v>
+      <c r="I4"/>
+      <c r="J4" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -807,8 +892,9 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="56.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="21.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="11.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="11.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="21.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -816,290 +902,374 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>12</v>
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="n">
         <v>2414.90776557478</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" t="n">
         <v>169</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="n">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" t="n">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" t="n">
         <v>0.799273820730713</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" t="n">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="n">
         <v>0.77433151443098</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" t="n">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" t="n">
         <v>0.104799671402601</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" t="n">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="n">
         <v>0.101116289167308</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" t="n">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" t="n">
         <v>0.108525944325693</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" t="n">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" t="n">
         <v>0.0887555412835664</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" t="n">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" t="n">
         <v>1209.08316155426</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" t="n">
         <v>48</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" t="n">
+        <v>11</v>
+      </c>
+      <c r="C13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" t="n">
+        <v>11</v>
+      </c>
+      <c r="C14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" t="n">
         <v>0.836739825992563</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" t="n">
+        <v>11</v>
+      </c>
+      <c r="C15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" t="n">
         <v>0.775517260739775</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
-      </c>
-      <c r="C16" t="n">
+        <v>11</v>
+      </c>
+      <c r="C16" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" t="n">
         <v>0.14138989096265</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>19</v>
-      </c>
-      <c r="C17" t="n">
+        <v>11</v>
+      </c>
+      <c r="C17" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17" t="n">
         <v>0.134554160355198</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
-      </c>
-      <c r="C18" t="n">
+        <v>11</v>
+      </c>
+      <c r="C18" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" t="n">
         <v>0.148342070924484</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>21</v>
-      </c>
-      <c r="C19" t="n">
+        <v>11</v>
+      </c>
+      <c r="C19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" t="n">
         <v>0.0792429984690142</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B20" t="s">
-        <v>13</v>
-      </c>
-      <c r="C20"/>
+        <v>11</v>
+      </c>
+      <c r="C20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20"/>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>14</v>
-      </c>
-      <c r="C21"/>
+        <v>11</v>
+      </c>
+      <c r="C21" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21"/>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B22" t="s">
-        <v>15</v>
-      </c>
-      <c r="C22"/>
+        <v>11</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22"/>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>16</v>
-      </c>
-      <c r="C23"/>
+        <v>11</v>
+      </c>
+      <c r="C23" t="s">
+        <v>21</v>
+      </c>
+      <c r="D23"/>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C24"/>
+        <v>11</v>
+      </c>
+      <c r="C24" t="s">
+        <v>22</v>
+      </c>
+      <c r="D24"/>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B25" t="s">
-        <v>18</v>
-      </c>
-      <c r="C25"/>
+        <v>11</v>
+      </c>
+      <c r="C25" t="s">
+        <v>23</v>
+      </c>
+      <c r="D25"/>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B26" t="s">
-        <v>19</v>
-      </c>
-      <c r="C26"/>
+        <v>11</v>
+      </c>
+      <c r="C26" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26"/>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B27" t="s">
-        <v>20</v>
-      </c>
-      <c r="C27"/>
+        <v>11</v>
+      </c>
+      <c r="C27" t="s">
+        <v>25</v>
+      </c>
+      <c r="D27"/>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B28" t="s">
-        <v>21</v>
-      </c>
-      <c r="C28"/>
+        <v>11</v>
+      </c>
+      <c r="C28" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1116,12 +1286,13 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="56.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="17.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="11.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="17.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="20.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="11.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="11.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="17.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="20.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="14.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1129,757 +1300,856 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G1" t="s">
-        <v>27</v>
+        <v>31</v>
+      </c>
+      <c r="H1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" t="n">
+        <v>33</v>
+      </c>
+      <c r="D2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" t="n">
         <v>0.432933956687998</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>0.0232522154997631</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>18.6190411271738</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D3" t="n">
+        <v>33</v>
+      </c>
+      <c r="D3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" t="n">
         <v>0.609984807423314</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>0.0182963331903839</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>33.3391833804113</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D4" t="n">
+        <v>33</v>
+      </c>
+      <c r="D4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" t="n">
         <v>0.582551376367235</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>0.0193394759188678</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>30.1223972568404</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" t="n">
+        <v>33</v>
+      </c>
+      <c r="D5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" t="n">
         <v>0.497719540906334</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>0.0231383749581501</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>21.5105659669942</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
         <v>33</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" t="n">
         <v>0.699499588906772</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>0.0157533842062468</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>44.4031314001341</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" t="n">
+        <v>33</v>
+      </c>
+      <c r="D7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" t="n">
         <v>0.702175925169589</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>0.01609526247015</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>43.6262488090414</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" t="n">
+        <v>33</v>
+      </c>
+      <c r="D8" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" t="n">
         <v>0.711361132396632</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>0.0150747401313164</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>47.188948280365</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" t="n">
+        <v>33</v>
+      </c>
+      <c r="D9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" t="n">
         <v>0.494823631078108</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>0.020775917604736</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>23.8171733490755</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" t="n">
+        <v>33</v>
+      </c>
+      <c r="D10" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" t="n">
         <v>0.676110719225227</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>0.0175016889004508</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>38.6311700014171</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>38</v>
-      </c>
-      <c r="D11" t="n">
+        <v>33</v>
+      </c>
+      <c r="D11" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" t="n">
         <v>0.521482517932356</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>0.0207394713004811</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>25.1444460843251</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
-      </c>
-      <c r="D12" t="n">
+        <v>33</v>
+      </c>
+      <c r="D12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E12" t="n">
         <v>0.634527014704012</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>0.0174104595811481</v>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>36.4451616998711</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>40</v>
-      </c>
-      <c r="D13" t="n">
+        <v>33</v>
+      </c>
+      <c r="D13" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" t="n">
         <v>0.715152776791424</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>0.0148349617922434</v>
       </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>48.2072543769779</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="C14" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" t="n">
+        <v>46</v>
+      </c>
+      <c r="D14" t="s">
+        <v>47</v>
+      </c>
+      <c r="E14" t="n">
         <v>0.493126754833674</v>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>0.0230633257532909</v>
       </c>
-      <c r="F14" t="n">
+      <c r="G14" t="n">
         <v>21.3814243491449</v>
       </c>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="C15" t="s">
-        <v>43</v>
-      </c>
-      <c r="D15" t="n">
+        <v>46</v>
+      </c>
+      <c r="D15" t="s">
+        <v>48</v>
+      </c>
+      <c r="E15" t="n">
         <v>0.475679524975317</v>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>0.0237677479647444</v>
       </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>20.0136557187038</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="C16" t="s">
-        <v>44</v>
-      </c>
-      <c r="D16" t="n">
+        <v>46</v>
+      </c>
+      <c r="D16" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" t="n">
         <v>0.726972809026527</v>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>0.0165182961783211</v>
       </c>
-      <c r="F16" t="n">
+      <c r="G16" t="n">
         <v>44.010157051223</v>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="C17" t="s">
-        <v>45</v>
-      </c>
-      <c r="D17" t="n">
+        <v>46</v>
+      </c>
+      <c r="D17" t="s">
+        <v>50</v>
+      </c>
+      <c r="E17" t="n">
         <v>0.56673050373625</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>0.0213764058480021</v>
       </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>26.5119640675806</v>
       </c>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="C18" t="s">
         <v>46</v>
       </c>
-      <c r="D18" t="n">
+      <c r="D18" t="s">
+        <v>51</v>
+      </c>
+      <c r="E18" t="n">
         <v>0.722974510005654</v>
       </c>
-      <c r="E18" t="n">
+      <c r="F18" t="n">
         <v>0.0169796408709362</v>
       </c>
-      <c r="F18" t="n">
+      <c r="G18" t="n">
         <v>42.578904671839</v>
       </c>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B19" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="C19" t="s">
-        <v>47</v>
-      </c>
-      <c r="D19" t="n">
+        <v>46</v>
+      </c>
+      <c r="D19" t="s">
+        <v>52</v>
+      </c>
+      <c r="E19" t="n">
         <v>0.591772629636741</v>
       </c>
-      <c r="E19" t="n">
+      <c r="F19" t="n">
         <v>0.0190029156465204</v>
       </c>
-      <c r="F19" t="n">
+      <c r="G19" t="n">
         <v>31.1411491080896</v>
       </c>
-      <c r="G19" t="n">
+      <c r="H19" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="C20" t="s">
-        <v>48</v>
-      </c>
-      <c r="D20" t="n">
+        <v>46</v>
+      </c>
+      <c r="D20" t="s">
+        <v>53</v>
+      </c>
+      <c r="E20" t="n">
         <v>0.480551972334813</v>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
         <v>0.0218525979199221</v>
       </c>
-      <c r="F20" t="n">
+      <c r="G20" t="n">
         <v>21.990610640244</v>
       </c>
-      <c r="G20" t="n">
+      <c r="H20" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="C21" t="s">
-        <v>49</v>
-      </c>
-      <c r="D21" t="n">
+        <v>46</v>
+      </c>
+      <c r="D21" t="s">
+        <v>54</v>
+      </c>
+      <c r="E21" t="n">
         <v>0.475020546358612</v>
       </c>
-      <c r="E21" t="n">
+      <c r="F21" t="n">
         <v>0.0236974347129152</v>
       </c>
-      <c r="F21" t="n">
+      <c r="G21" t="n">
         <v>20.0452307227889</v>
       </c>
-      <c r="G21" t="n">
+      <c r="H21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="C22" t="s">
-        <v>51</v>
-      </c>
-      <c r="D22" t="n">
+        <v>55</v>
+      </c>
+      <c r="D22" t="s">
+        <v>56</v>
+      </c>
+      <c r="E22" t="n">
         <v>0.588396197791704</v>
       </c>
-      <c r="E22" t="n">
+      <c r="F22" t="n">
         <v>0.0213374819277609</v>
       </c>
-      <c r="F22" t="n">
+      <c r="G22" t="n">
         <v>27.5757092511548</v>
       </c>
-      <c r="G22" t="n">
+      <c r="H22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B23" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="C23" t="s">
-        <v>52</v>
-      </c>
-      <c r="D23" t="n">
+        <v>55</v>
+      </c>
+      <c r="D23" t="s">
+        <v>57</v>
+      </c>
+      <c r="E23" t="n">
         <v>-0.343365315596442</v>
       </c>
-      <c r="E23" t="n">
+      <c r="F23" t="n">
         <v>0.0270081692503478</v>
       </c>
-      <c r="F23" t="n">
+      <c r="G23" t="n">
         <v>-12.7133872871453</v>
       </c>
-      <c r="G23" t="n">
+      <c r="H23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="C24" t="s">
-        <v>53</v>
-      </c>
-      <c r="D24" t="n">
+        <v>55</v>
+      </c>
+      <c r="D24" t="s">
+        <v>58</v>
+      </c>
+      <c r="E24" t="n">
         <v>0.669224146244267</v>
       </c>
-      <c r="E24" t="n">
+      <c r="F24" t="n">
         <v>0.0186188313550063</v>
       </c>
-      <c r="F24" t="n">
+      <c r="G24" t="n">
         <v>35.9434023266087</v>
       </c>
-      <c r="G24" t="n">
+      <c r="H24" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B25" t="s">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="C25" t="s">
-        <v>55</v>
-      </c>
-      <c r="D25" t="n">
+        <v>59</v>
+      </c>
+      <c r="D25" t="s">
+        <v>60</v>
+      </c>
+      <c r="E25" t="n">
         <v>0.832956918786042</v>
       </c>
-      <c r="E25" t="n">
+      <c r="F25" t="n">
         <v>0.0156293179041361</v>
       </c>
-      <c r="F25" t="n">
+      <c r="G25" t="n">
         <v>53.2945150834517</v>
       </c>
-      <c r="G25" t="n">
+      <c r="H25" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B26" t="s">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="C26" t="s">
-        <v>56</v>
-      </c>
-      <c r="D26" t="n">
+        <v>59</v>
+      </c>
+      <c r="D26" t="s">
+        <v>61</v>
+      </c>
+      <c r="E26" t="n">
         <v>-0.274614928807825</v>
       </c>
-      <c r="E26" t="n">
+      <c r="F26" t="n">
         <v>0.0290647109570638</v>
       </c>
-      <c r="F26" t="n">
+      <c r="G26" t="n">
         <v>-9.44839703424208</v>
       </c>
-      <c r="G26" t="n">
+      <c r="H26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B27" t="s">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="C27" t="s">
-        <v>57</v>
-      </c>
-      <c r="D27" t="n">
+        <v>59</v>
+      </c>
+      <c r="D27" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" t="n">
         <v>0.754084669453953</v>
       </c>
-      <c r="E27" t="n">
+      <c r="F27" t="n">
         <v>0.018086601569778</v>
       </c>
-      <c r="F27" t="n">
+      <c r="G27" t="n">
         <v>41.6929994584498</v>
       </c>
-      <c r="G27" t="n">
+      <c r="H27" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B28" t="s">
-        <v>58</v>
+        <v>11</v>
       </c>
       <c r="C28" t="s">
-        <v>59</v>
-      </c>
-      <c r="D28" t="n">
+        <v>63</v>
+      </c>
+      <c r="D28" t="s">
+        <v>64</v>
+      </c>
+      <c r="E28" t="n">
         <v>0.704323694920484</v>
       </c>
-      <c r="E28" t="n">
+      <c r="F28" t="n">
         <v>0.0158989637544577</v>
       </c>
-      <c r="F28" t="n">
+      <c r="G28" t="n">
         <v>44.2999748787407</v>
       </c>
-      <c r="G28" t="n">
+      <c r="H28" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B29" t="s">
-        <v>58</v>
+        <v>11</v>
       </c>
       <c r="C29" t="s">
-        <v>60</v>
-      </c>
-      <c r="D29" t="n">
+        <v>63</v>
+      </c>
+      <c r="D29" t="s">
+        <v>65</v>
+      </c>
+      <c r="E29" t="n">
         <v>0.605373846977582</v>
       </c>
-      <c r="E29" t="n">
+      <c r="F29" t="n">
         <v>0.0201993022815593</v>
       </c>
-      <c r="F29" t="n">
+      <c r="G29" t="n">
         <v>29.9700375062088</v>
       </c>
-      <c r="G29" t="n">
+      <c r="H29" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B30" t="s">
-        <v>58</v>
+        <v>11</v>
       </c>
       <c r="C30" t="s">
-        <v>61</v>
-      </c>
-      <c r="D30" t="n">
+        <v>63</v>
+      </c>
+      <c r="D30" t="s">
+        <v>66</v>
+      </c>
+      <c r="E30" t="n">
         <v>0.707412097466206</v>
       </c>
-      <c r="E30" t="n">
+      <c r="F30" t="n">
         <v>0.016082400291344</v>
       </c>
-      <c r="F30" t="n">
+      <c r="G30" t="n">
         <v>43.9867236638149</v>
       </c>
-      <c r="G30" t="n">
+      <c r="H30" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B31" t="s">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="C31" t="s">
-        <v>63</v>
-      </c>
-      <c r="D31" t="n">
+        <v>67</v>
+      </c>
+      <c r="D31" t="s">
+        <v>68</v>
+      </c>
+      <c r="E31" t="n">
         <v>0.552517977481675</v>
       </c>
-      <c r="E31" t="n">
+      <c r="F31" t="n">
         <v>0.0278057205261411</v>
       </c>
-      <c r="F31" t="n">
+      <c r="G31" t="n">
         <v>19.87065852015</v>
       </c>
-      <c r="G31" t="n">
+      <c r="H31" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B32" t="s">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="C32" t="s">
-        <v>64</v>
-      </c>
-      <c r="D32" t="n">
+        <v>67</v>
+      </c>
+      <c r="D32" t="s">
+        <v>69</v>
+      </c>
+      <c r="E32" t="n">
         <v>0.0292154685707168</v>
       </c>
-      <c r="E32" t="n">
+      <c r="F32" t="n">
         <v>0.0327097379728803</v>
       </c>
-      <c r="F32" t="n">
+      <c r="G32" t="n">
         <v>0.893173421167098</v>
       </c>
-      <c r="G32" t="n">
+      <c r="H32" t="n">
         <v>0.371764309243827</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B33" t="s">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="C33" t="s">
-        <v>65</v>
-      </c>
-      <c r="D33" t="n">
+        <v>67</v>
+      </c>
+      <c r="D33" t="s">
+        <v>70</v>
+      </c>
+      <c r="E33" t="n">
         <v>0.621666656430318</v>
       </c>
-      <c r="E33" t="n">
+      <c r="F33" t="n">
         <v>0.0276852115640481</v>
       </c>
-      <c r="F33" t="n">
+      <c r="G33" t="n">
         <v>22.4548277332875</v>
       </c>
-      <c r="G33" t="n">
+      <c r="H33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1898,9 +2168,10 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="56.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="17.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="10.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="11.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="17.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="17.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1908,111 +2179,356 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>66</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D1" t="s">
-        <v>68</v>
+        <v>72</v>
+      </c>
+      <c r="E1" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" t="n">
-        <v>-0.0581517832749122</v>
+        <v>33</v>
+      </c>
+      <c r="D2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.769652845746389</v>
+        <v>46</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-0.0581517832749122</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>58</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>54</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.825060874717827</v>
+        <v>33</v>
+      </c>
+      <c r="D4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-0.0581517832749122</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>54</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.495282824303017</v>
+        <v>46</v>
+      </c>
+      <c r="D5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
-      </c>
-      <c r="D6" t="n">
-        <v>1.03945393775832</v>
+        <v>55</v>
+      </c>
+      <c r="D6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.836716546106013</v>
+        <v>59</v>
+      </c>
+      <c r="D7" t="s">
+        <v>55</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.769652845746389</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>62</v>
-      </c>
-      <c r="D8" t="n">
+        <v>63</v>
+      </c>
+      <c r="D8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1.03945393775832</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>67</v>
+      </c>
+      <c r="D9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9" t="n">
         <v>0.804916632569058</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.769652845746389</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" t="s">
+        <v>59</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>63</v>
+      </c>
+      <c r="D12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.825060874717827</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.495282824303017</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" t="s">
+        <v>63</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1.03945393775832</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" t="s">
+        <v>63</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.825060874717827</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" t="s">
+        <v>63</v>
+      </c>
+      <c r="D16" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" t="s">
+        <v>67</v>
+      </c>
+      <c r="D17" t="s">
+        <v>63</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.836716546106013</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>12</v>
+      </c>
+      <c r="B18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.804916632569058</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" t="s">
+        <v>59</v>
+      </c>
+      <c r="D19" t="s">
+        <v>67</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.495282824303017</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" t="s">
+        <v>63</v>
+      </c>
+      <c r="D20" t="s">
+        <v>67</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.836716546106013</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" t="s">
+        <v>67</v>
+      </c>
+      <c r="D21" t="s">
+        <v>67</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2040,21 +2556,21 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C1" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D1" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C2" t="n">
         <v>0.860913531820943</v>
@@ -2065,10 +2581,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C3" t="n">
         <v>0.775201716778637</v>
@@ -2076,6 +2592,22 @@
       <c r="D3" t="n">
         <v>0.356572887171823</v>
       </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4"/>
+      <c r="C4"/>
+      <c r="D4"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5"/>
+      <c r="C5"/>
+      <c r="D5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2094,74 +2626,82 @@
     <col min="1" max="1" width="32.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="10.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="5.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="12.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="27.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="11.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="10.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="17.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="29.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="20.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="12.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="14.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="10.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="17.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="29.71" hidden="0" customWidth="1"/>
     <col min="12" max="12" width="20.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="22.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="12.71" hidden="0" customWidth="1"/>
     <col min="14" max="14" width="20.71" hidden="0" customWidth="1"/>
-    <col min="15" max="15" width="14.71" hidden="0" customWidth="1"/>
-    <col min="16" max="16" width="120.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="22.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="20.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="14.71" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="95.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B1" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C1" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D1" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E1" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F1" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="G1" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H1" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="I1" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="J1" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="K1" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="L1" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="M1" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="N1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="O1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="P1" t="s">
-        <v>86</v>
+        <v>91</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>92</v>
+      </c>
+      <c r="R1" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B2" t="n">
         <v>1211</v>
@@ -2170,31 +2710,31 @@
         <v>20</v>
       </c>
       <c r="D2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F2" t="n">
         <v>0.874681143514216</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
         <v>8143.4905069051</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>190</v>
       </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
         <v>0.556795490374051</v>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
         <v>0.618750772837551</v>
       </c>
-      <c r="J2" t="n">
+      <c r="L2" t="n">
         <v>60.55</v>
-      </c>
-      <c r="K2" t="b">
-        <v>1</v>
-      </c>
-      <c r="L2" t="b">
-        <v>1</v>
       </c>
       <c r="M2" t="b">
         <v>1</v>
@@ -2205,13 +2745,19 @@
       <c r="O2" t="b">
         <v>1</v>
       </c>
-      <c r="P2" t="s">
-        <v>88</v>
+      <c r="P2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="b">
+        <v>1</v>
+      </c>
+      <c r="R2" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="B3" t="n">
         <v>1211</v>
@@ -2220,31 +2766,31 @@
         <v>12</v>
       </c>
       <c r="D3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F3" t="n">
         <v>0.836508465500397</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
         <v>4335.52993751679</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>66</v>
       </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
         <v>0.776886802110134</v>
       </c>
-      <c r="I3" t="n">
+      <c r="K3" t="n">
         <v>0.645536890534378</v>
       </c>
-      <c r="J3" t="n">
+      <c r="L3" t="n">
         <v>100.916666666667</v>
-      </c>
-      <c r="K3" t="b">
-        <v>1</v>
-      </c>
-      <c r="L3" t="b">
-        <v>1</v>
       </c>
       <c r="M3" t="b">
         <v>1</v>
@@ -2255,8 +2801,14 @@
       <c r="O3" t="b">
         <v>1</v>
       </c>
-      <c r="P3" t="s">
-        <v>88</v>
+      <c r="P3" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="b">
+        <v>1</v>
+      </c>
+      <c r="R3" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>